<commit_message>
Add full question generation pipeline and all model responses
- Add generate_responses.py: automated API runner for Claude (claude-sonnet-4-6),
  ChatGPT (gpt-4o-2024-11-20), Gemini (gemini-2.5-flash), and Groq (llama-3.3-70b-versatile)
- Fix DATA_INTERP_TEMPLATE: Output Format section was placed after the second ---
  separator and was being stripped before API calls, causing all Cat 2 batches to
  return markdown instead of JSON across all models
- Add .env.example with all four API key placeholders
- Add prompt.md and response.json for all 28 batches × 4 models (113 files total)
- Standardise generated_by field to exact model ID strings across all responses
- Update section_list.xlsx and passages/cat7_batch2.txt

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/section_list.xlsx
+++ b/section_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Aiden/Desktop/portfolio/climate_benchmarking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAEB73F5-F74A-6E49-ADEB-29410A21A5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{620BCE4D-B796-C142-BD94-523BE6CBE026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1720" yWindow="1400" windowWidth="33720" windowHeight="19700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4480" yWindow="1400" windowWidth="31360" windowHeight="19700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Section List" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="191">
   <si>
     <t>batch_id</t>
   </si>
@@ -588,6 +588,12 @@
   </si>
   <si>
     <t>IPCC AR6 WG1 Chapter 2 Section 2.3.1.1.3</t>
+  </si>
+  <si>
+    <t>2.4.3.2.1</t>
+  </si>
+  <si>
+    <t>IPCC AR6 WG2 Chapter 2 Section 2.4.3.2.1</t>
   </si>
 </sst>
 </file>
@@ -607,15 +613,18 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1908,11 +1917,11 @@
       <c r="E28" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F28" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>164</v>
+      <c r="F28" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>190</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>17</v>

</xml_diff>